<commit_message>
fix: arena reads "Engagement", matching the one-pager
Column B took the arena names verbatim from the 19 Aug workbook's
Module column, which spells the third one "Patient Engagement". The
vendor one-pager and the questionnaire's Part B both say "Engagement".
Renamed on the sheet, the drop-down list and the Start Here counts:
34 Capacity Management / 29 Scheduling Engine / 25 Engagement.

Left alone deliberately: the source documents that record the original
DE-02 wording (whiteboard session, discovery notes) and the workbook's
own Module column upstream. This is a display name, not a placement
change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MErRq7TByJ5fbijWwJSpv1
</commit_message>
<xml_diff>
--- a/agents/compassus-capacity-pm/artifacts/Capacity-Scheduling-Variable-Workbook.xlsx
+++ b/agents/compassus-capacity-pm/artifacts/Capacity-Scheduling-Variable-Workbook.xlsx
@@ -1033,7 +1033,7 @@
     <row r="33">
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="D33" s="12">
-        <f>COUNTIF('Master List'!$B$2:$B$89,"Patient Engagement")</f>
+        <f>COUNTIF('Master List'!$B$2:$B$89,"Engagement")</f>
         <v/>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
         </is>
       </c>
       <c r="D44" s="12">
-        <f>COUNTIFS('Master List'!$O$2:$O$89,"Drifts*",'Master List'!$B$2:$B$89,"&lt;&gt;Patient Engagement")</f>
+        <f>COUNTIFS('Master List'!$O$2:$O$89,"Drifts*",'Master List'!$B$2:$B$89,"&lt;&gt;Engagement")</f>
         <v/>
       </c>
     </row>
@@ -8338,7 +8338,7 @@
       </c>
       <c r="B65" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C65" s="18" t="inlineStr">
@@ -8445,7 +8445,7 @@
       </c>
       <c r="B66" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C66" s="18" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="B67" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C67" s="18" t="inlineStr"/>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="B68" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C68" s="18" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="B69" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C69" s="18" t="inlineStr">
@@ -8869,7 +8869,7 @@
       </c>
       <c r="B70" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C70" s="18" t="inlineStr">
@@ -8976,7 +8976,7 @@
       </c>
       <c r="B71" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C71" s="18" t="inlineStr">
@@ -9083,7 +9083,7 @@
       </c>
       <c r="B72" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C72" s="18" t="inlineStr"/>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="B73" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -9293,7 +9293,7 @@
       </c>
       <c r="B74" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C74" s="18" t="inlineStr"/>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="B75" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C75" s="18" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="B76" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C76" s="18" t="inlineStr">
@@ -9610,7 +9610,7 @@
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C77" s="18" t="inlineStr"/>
@@ -9713,7 +9713,7 @@
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C78" s="18" t="inlineStr"/>
@@ -9816,7 +9816,7 @@
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C79" s="18" t="inlineStr"/>
@@ -9919,7 +9919,7 @@
       </c>
       <c r="B80" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C80" s="18" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C81" s="18" t="inlineStr"/>
@@ -10129,7 +10129,7 @@
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C82" s="18" t="inlineStr"/>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C83" s="18" t="inlineStr">
@@ -10339,7 +10339,7 @@
       </c>
       <c r="B84" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C84" s="18" t="inlineStr">
@@ -10446,7 +10446,7 @@
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C85" s="18" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="E85" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Patient Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F85" s="18" t="inlineStr">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C86" s="18" t="inlineStr">
@@ -10660,7 +10660,7 @@
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C87" s="18" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Patient Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F87" s="18" t="inlineStr">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B88" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C88" s="18" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Patient Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F88" s="18" t="inlineStr">
@@ -10874,7 +10874,7 @@
       </c>
       <c r="B89" s="25" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="C89" s="18" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Patient Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F89" s="18" t="inlineStr">
@@ -11210,7 +11210,7 @@
     <row r="4">
       <c r="A4" s="27" t="inlineStr">
         <is>
-          <t>Patient Engagement</t>
+          <t>Engagement</t>
         </is>
       </c>
       <c r="B4" s="27" t="inlineStr">

</xml_diff>

<commit_message>
revert: keep "Scheduling Engine" -- Colin's call
Column B is Capacity Management / Scheduling Engine / Engagement.
"Patient Engagement" -> "Engagement" stands; the Scheduling rename does
not. Restores the arena naming from ba6d758 and re-applies the
Engagement definition on top of it, so the sheet still says what
engagement covers -- office to clinician, clinician to office, clinician
to clinician, care team to each other, patient and caregiver.

The workbook's Module column now differs from this sheet on one label
only, which the ledger records.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MErRq7TByJ5fbijWwJSpv1
</commit_message>
<xml_diff>
--- a/agents/compassus-capacity-pm/artifacts/Capacity-Scheduling-Variable-Workbook.xlsx
+++ b/agents/compassus-capacity-pm/artifacts/Capacity-Scheduling-Variable-Workbook.xlsx
@@ -786,7 +786,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>One of the three project categories: Capacity Management, Scheduling, Engagement. Placement is straight from the Module column of the 19 Aug workbook, which is authoritative — change it there, not here. Only the names are shortened to match the one-pager (the workbook writes the third one as “Patient Engagement”).</t>
+          <t>One of the three project categories: Capacity Management, Scheduling Engine, Engagement. Placement is straight from the Module column of the 19 Aug workbook, which is authoritative — change it there, not here. The only renaming is “Patient Engagement” → “Engagement”, to match the one-pager.</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Not only the patient. Engagement is the contact work that turns a schedule into delivered visits, whoever it is with — office to clinician, clinician back to the office, clinician to clinician, and the care team to each other, as well as the patient and their caregiver. Finding coverage for a call-out is engagement; so is keeping the case manager in step. The one-pager already says so: “with patients, clinicians and the office.”</t>
+          <t>Not only the patient — which is exactly why the label was shortened. Engagement is the contact work that turns a schedule into delivered visits, whoever it is with: office to clinician, clinician back to the office, clinician to clinician, and the care team to each other, as well as the patient and their caregiver. Finding coverage for a call-out is engagement; so is keeping the case manager in step. The one-pager already says so: “with patients, clinicians and the office.”</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1017,7 @@
     <row r="32">
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -1026,7 +1026,7 @@
         </is>
       </c>
       <c r="D32" s="12">
-        <f>COUNTIF('Master List'!$B$2:$B$89,"Scheduling")</f>
+        <f>COUNTIF('Master List'!$B$2:$B$89,"Scheduling Engine")</f>
         <v/>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F28" s="18" t="inlineStr">
@@ -4581,7 +4581,7 @@
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -4684,7 +4684,7 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="E35" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F35" s="18" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B36" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="B37" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr"/>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr"/>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="B41" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr"/>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="B42" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="B43" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr"/>
@@ -6131,7 +6131,7 @@
       </c>
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
@@ -6238,7 +6238,7 @@
       </c>
       <c r="B45" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr"/>
@@ -6341,7 +6341,7 @@
       </c>
       <c r="B46" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
@@ -6448,7 +6448,7 @@
       </c>
       <c r="B47" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr"/>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="B48" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr"/>
@@ -6654,7 +6654,7 @@
       </c>
       <c r="B49" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C49" s="18" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="B50" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C50" s="18" t="inlineStr"/>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="B51" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C51" s="18" t="inlineStr"/>
@@ -6967,7 +6967,7 @@
       </c>
       <c r="B52" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C52" s="18" t="inlineStr"/>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="B53" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C53" s="18" t="inlineStr"/>
@@ -7173,7 +7173,7 @@
       </c>
       <c r="B54" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C54" s="18" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="B55" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C55" s="18" t="inlineStr">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="B56" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C56" s="18" t="inlineStr"/>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="B57" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C57" s="18" t="inlineStr">
@@ -7597,7 +7597,7 @@
       </c>
       <c r="B58" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C58" s="18" t="inlineStr"/>
@@ -7700,7 +7700,7 @@
       </c>
       <c r="B59" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C59" s="18" t="inlineStr">
@@ -7807,7 +7807,7 @@
       </c>
       <c r="B60" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C60" s="18" t="inlineStr">
@@ -7914,7 +7914,7 @@
       </c>
       <c r="B61" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C61" s="18" t="inlineStr">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="B62" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C62" s="18" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="B63" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C63" s="18" t="inlineStr"/>
@@ -8231,7 +8231,7 @@
       </c>
       <c r="B64" s="24" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="C64" s="18" t="inlineStr">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="E65" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F65" s="18" t="inlineStr">
@@ -8460,7 +8460,7 @@
       </c>
       <c r="E66" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F66" s="18" t="inlineStr">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="E67" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F67" s="18" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="E68" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F68" s="18" t="inlineStr">
@@ -8777,7 +8777,7 @@
       </c>
       <c r="E69" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F69" s="18" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="E70" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F70" s="18" t="inlineStr">
@@ -8991,7 +8991,7 @@
       </c>
       <c r="E71" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F71" s="18" t="inlineStr">
@@ -9094,7 +9094,7 @@
       </c>
       <c r="E72" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F72" s="18" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="E73" s="23" t="inlineStr">
         <is>
-          <t>Differs — the one-pager groups this under Scheduling</t>
+          <t>Differs — the one-pager groups this under Scheduling Engine</t>
         </is>
       </c>
       <c r="F73" s="18" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="E85" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F85" s="18" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F87" s="18" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F88" s="18" t="inlineStr">
@@ -10889,7 +10889,7 @@
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling; write this back to the workbook</t>
+          <t>Ruled 25 Aug — moved to Engagement. The 8.19 workbook still has it under Scheduling Engine; write this back to the workbook</t>
         </is>
       </c>
       <c r="F89" s="18" t="inlineStr">
@@ -11158,7 +11158,7 @@
     <row r="3">
       <c r="A3" s="27" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Scheduling Engine</t>
         </is>
       </c>
       <c r="B3" s="27" t="inlineStr">

</xml_diff>